<commit_message>
List and Sets Done
</commit_message>
<xml_diff>
--- a/learning_summary.xlsx
+++ b/learning_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mohsin-Personal\Python-Learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC81A23-F2FD-4B1C-A664-3C1BDC34DE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B39B935-9928-440A-BFC8-B2468ECA4691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{975AB781-A782-4B7B-AE97-21F5DA85B194}"/>
   </bookViews>
@@ -284,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -299,14 +299,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,16 +638,16 @@
       </c>
     </row>
     <row r="2" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="7"/>
+      <c r="B2" s="9"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
     </row>
@@ -654,7 +655,7 @@
       <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="7" t="s">
         <v>3</v>
       </c>
     </row>
@@ -702,7 +703,7 @@
       <c r="A10" s="4">
         <v>8</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="10" t="s">
         <v>9</v>
       </c>
     </row>
@@ -747,10 +748,10 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="7"/>
+      <c r="B16" s="9"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
@@ -825,16 +826,16 @@
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="7"/>
+      <c r="B26" s="9"/>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>1</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="6" t="s">
         <v>27</v>
       </c>
     </row>
@@ -842,7 +843,7 @@
       <c r="A28" s="4">
         <v>2</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="6" t="s">
         <v>28</v>
       </c>
     </row>
@@ -850,7 +851,7 @@
       <c r="A29" s="4">
         <v>3</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="6" t="s">
         <v>29</v>
       </c>
     </row>
@@ -858,7 +859,7 @@
       <c r="A30" s="4">
         <v>4</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="6" t="s">
         <v>30</v>
       </c>
     </row>
@@ -866,7 +867,7 @@
       <c r="A31" s="4">
         <v>5</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="6" t="s">
         <v>31</v>
       </c>
     </row>

</xml_diff>

<commit_message>
operators done, bitwise operators are left will be done later.
</commit_message>
<xml_diff>
--- a/learning_summary.xlsx
+++ b/learning_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Mohsin-Personal\Python-Learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9CFA20-6E78-44C5-A91D-C6CD8A2129C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590CDD00-CFF3-4FF2-8372-31E118CFDAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{975AB781-A782-4B7B-AE97-21F5DA85B194}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="44">
   <si>
     <t>S#</t>
   </si>
@@ -186,7 +186,37 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>.encode() method left as this is very importance method and need to be practiced more than other methods</t>
+    <t>There are a lot of string methods which can be learn day by day. So I'm moving on for now.</t>
+  </si>
+  <si>
+    <t>Bitwise operators are left.</t>
+  </si>
+  <si>
+    <t>Bitwise Conditionals are left.</t>
+  </si>
+  <si>
+    <t>Bitwise loops are left.</t>
+  </si>
+  <si>
+    <t>Bitwise Functions are left.</t>
+  </si>
+  <si>
+    <t>Bitwise scope are left.</t>
+  </si>
+  <si>
+    <t>Bitwise Lists are left.</t>
+  </si>
+  <si>
+    <t>Bitwise tuples are left.</t>
+  </si>
+  <si>
+    <t>Bitwise dictionaries are left.</t>
+  </si>
+  <si>
+    <t>Bitwise sets are left.</t>
+  </si>
+  <si>
+    <t>Bitwise File I/O are left.</t>
   </si>
 </sst>
 </file>
@@ -305,29 +335,29 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -647,7 +677,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="61.33203125" style="11" customWidth="1"/>
+    <col min="2" max="2" width="61.33203125" style="8" customWidth="1"/>
     <col min="3" max="3" width="40.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -655,25 +685,25 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="12" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="7"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="13"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="9" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1"/>
@@ -682,7 +712,7 @@
       <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="1"/>
@@ -694,13 +724,15 @@
       <c r="B5" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="1"/>
+      <c r="C5" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="1"/>
@@ -709,7 +741,7 @@
       <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="6" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="1"/>
@@ -718,7 +750,7 @@
       <c r="A8" s="4">
         <v>6</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="1"/>
@@ -727,7 +759,7 @@
       <c r="A9" s="4">
         <v>7</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="1"/>
@@ -736,7 +768,7 @@
       <c r="A10" s="4">
         <v>8</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="1"/>
@@ -745,7 +777,7 @@
       <c r="A11" s="4">
         <v>9</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C11" s="1"/>
@@ -754,7 +786,7 @@
       <c r="A12" s="4">
         <v>10</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C12" s="1"/>
@@ -763,19 +795,19 @@
       <c r="A13" s="4">
         <v>11</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="9" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>12</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="10" t="s">
         <v>33</v>
       </c>
     </row>
@@ -783,23 +815,23 @@
       <c r="A15" s="4">
         <v>13</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="1"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="5"/>
+      <c r="B16" s="11"/>
       <c r="C16" s="1"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>1</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C17" s="1"/>
@@ -808,7 +840,7 @@
       <c r="A18" s="4">
         <v>2</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C18" s="1"/>
@@ -817,7 +849,7 @@
       <c r="A19" s="4">
         <v>3</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C19" s="1"/>
@@ -826,7 +858,7 @@
       <c r="A20" s="4">
         <v>4</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="1"/>
@@ -835,7 +867,7 @@
       <c r="A21" s="4">
         <v>5</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C21" s="1"/>
@@ -844,7 +876,7 @@
       <c r="A22" s="4">
         <v>6</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C22" s="1"/>
@@ -853,7 +885,7 @@
       <c r="A23" s="4">
         <v>7</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C23" s="1"/>
@@ -862,7 +894,7 @@
       <c r="A24" s="4">
         <v>8</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="6" t="s">
         <v>24</v>
       </c>
       <c r="C24" s="1"/>
@@ -871,23 +903,23 @@
       <c r="A25" s="4">
         <v>9</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C25" s="1"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="5"/>
+      <c r="B26" s="11"/>
       <c r="C26" s="1"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>1</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C27" s="1"/>
@@ -896,7 +928,7 @@
       <c r="A28" s="4">
         <v>2</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="7" t="s">
         <v>28</v>
       </c>
       <c r="C28" s="1"/>
@@ -905,7 +937,7 @@
       <c r="A29" s="4">
         <v>3</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="7" t="s">
         <v>29</v>
       </c>
       <c r="C29" s="1"/>
@@ -914,7 +946,7 @@
       <c r="A30" s="4">
         <v>4</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="7" t="s">
         <v>30</v>
       </c>
       <c r="C30" s="1"/>
@@ -923,7 +955,7 @@
       <c r="A31" s="4">
         <v>5</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="7" t="s">
         <v>31</v>
       </c>
       <c r="C31" s="1"/>

</xml_diff>